<commit_message>
docs: decisões D16-D23, dados reais x simulados, DER lógico, fluxograma do caixa, requisitos e rastreabilidade atualizados
</commit_message>
<xml_diff>
--- a/docs/requisitos/requisitos.xlsx
+++ b/docs/requisitos/requisitos.xlsx
@@ -1025,12 +1025,12 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Cada terminal (BALCAO, DELIVERY) abre e fecha caixa por dia, com valor de abertura, valor contado no fechamento e responsáveis; todo pagamento é lançado em um caixa; a diferença entre o contado e o esperado em dinheiro é auditável.</t>
+          <t>O terminal (na fita: "Mont Ararat Delivery", que registra vendas de mesa, balcão e delivery) abre e fecha o turno com valor de abertura, valor de fechamento informado e responsáveis; todo pagamento é lançado em um caixa; os recebimentos são agrupados em dinheiro, cartão e outras formas; a diferença de caixa = fechamento − (abertura + soma de recebimentos) é auditável, e o fechamento mostra serviço de mesa, tickets e cancelamentos de mesa.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>NOVO: baseado no relatório de fechamento de caixa da Evidência 1 do grupo.</t>
+          <t>NOVO: baseado na fita de fechamento de turno real (Evidência 1 do grupo), lida campo a campo.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1040,12 +1040,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Auditoria AUD03.</t>
+          <t>Consulta G14 (reproduz a fita); auditoria AUD03 e AUD11; teste T43.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>caixa, pagamento.id_caixa</t>
+          <t>caixa, pagamento.id_caixa, forma_pagamento.grupo_fechamento, pedido.valor_servico, item_pedido.cancelado</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>39 testes de restrição (sql/testes) com controles positivos.</t>
+          <t>43 testes de restrição (sql/testes) com controles positivos.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Produto marcado como montagem_especial não pode ser incluído em pedido DELIVERY.</t>
+          <t>Produto marcado como montagem_especial (na massa: Dilúvio, assumido; decisão D13) não pode ser incluído em pedido DELIVERY, nem diretamente nem dentro de um combo.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1722,12 +1722,12 @@
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Trigger trg_item_pedido_bi; testes T13-T14.</t>
+          <t>Triggers trg_item_pedido_bi e trg_item_combo_pedido_bi; testes T13-T14 e T40-T41.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>produto.montagem_especial, trg_item_pedido_bi</t>
+          <t>produto.montagem_especial, trg_item_pedido_bi, trg_item_combo_pedido_bi</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2038,7 @@
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Massa contém reajuste do Dois Dilúvios em 01/10/2026.</t>
+          <t>Massa contém reajuste fictício do Dilúvio em 01/10/2026 (D18).</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">

</xml_diff>